<commit_message>
Tests actualizados de app y web
</commit_message>
<xml_diff>
--- a/App/TestCases_App/User_Home.xlsx
+++ b/App/TestCases_App/User_Home.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\App\TestCases_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F106DA59-5966-432C-95C8-AD1E3635D1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA225306-2EB6-44A6-AF0A-38344A991E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>Num</t>
   </si>
@@ -172,6 +172,19 @@
   <si>
     <t>_ Al pulsar para teclear el email, el teclado tapa los campos. Se deben desplazar hacia arriba para que el usuario vea que valores introduce en el correo eletrónico y en la contraseña.userh001.jpg
 _ Se debe cambiar además "email" por "correo electrónico"</t>
+  </si>
+  <si>
+    <t>USERH000</t>
+  </si>
+  <si>
+    <t>Las etiquetas de todos los usuarios pone "Camarero": home_users.jpg</t>
+  </si>
+  <si>
+    <t>Select an user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select an user
+</t>
   </si>
 </sst>
 </file>
@@ -609,14 +622,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="41.5703125" customWidth="1"/>
     <col min="5" max="6" width="33.42578125" customWidth="1"/>
-    <col min="8" max="8" width="91.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="66.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -645,94 +658,92 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>25</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F2" s="3"/>
       <c r="G2" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H2" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>26</v>
-      </c>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>24</v>
@@ -747,42 +758,44 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="7"/>
+      <c r="H6" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>30</v>
@@ -795,66 +808,66 @@
       </c>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" s="5" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>12</v>
       </c>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" s="5" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>12</v>
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>24</v>
@@ -867,9 +880,33 @@
       </c>
       <c r="H10" s="7"/>
     </row>
+    <row r="11" spans="1:8" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G10">
+  <conditionalFormatting sqref="G2:G11">
     <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PTE">
       <formula>NOT(ISERROR(SEARCH("PTE",G2)))</formula>
     </cfRule>

</xml_diff>